<commit_message>
Refresh the corpus workbook and update the changelog and handoff for a fresh chat
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/corpus/corpus.xlsx
+++ b/corpus/corpus.xlsx
@@ -695,7 +695,7 @@
       <c r="AA2" s="3" t="n"/>
       <c r="AB2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       <c r="AA3" s="3" t="n"/>
       <c r="AB3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       <c r="AA4" s="3" t="n"/>
       <c r="AB4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       <c r="AA5" s="3" t="n"/>
       <c r="AB5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -1063,7 +1063,7 @@
       <c r="AA6" s="3" t="n"/>
       <c r="AB6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -1153,7 +1153,7 @@
       <c r="AA7" s="3" t="n"/>
       <c r="AB7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       <c r="AA8" s="3" t="n"/>
       <c r="AB8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -1333,7 +1333,7 @@
       <c r="AA9" s="3" t="n"/>
       <c r="AB9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -1423,7 +1423,7 @@
       <c r="AA10" s="3" t="n"/>
       <c r="AB10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -1513,7 +1513,7 @@
       <c r="AA11" s="3" t="n"/>
       <c r="AB11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -1611,7 +1611,7 @@
       <c r="AA12" s="3" t="n"/>
       <c r="AB12" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -1701,7 +1701,7 @@
       <c r="AA13" s="3" t="n"/>
       <c r="AB13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -1799,7 +1799,7 @@
       <c r="AA14" s="3" t="n"/>
       <c r="AB14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
       <c r="AA15" s="3" t="n"/>
       <c r="AB15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -1983,7 +1983,7 @@
       <c r="AA16" s="3" t="n"/>
       <c r="AB16" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -2077,7 +2077,7 @@
       <c r="AA17" s="3" t="n"/>
       <c r="AB17" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
       <c r="AA18" s="3" t="n"/>
       <c r="AB18" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -2269,7 +2269,7 @@
       <c r="AA19" s="3" t="n"/>
       <c r="AB19" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -2363,7 +2363,7 @@
       <c r="AA20" s="3" t="n"/>
       <c r="AB20" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -2461,7 +2461,7 @@
       <c r="AA21" s="3" t="n"/>
       <c r="AB21" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -2559,7 +2559,7 @@
       <c r="AA22" s="3" t="n"/>
       <c r="AB22" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -2645,7 +2645,7 @@
       <c r="AA23" s="3" t="n"/>
       <c r="AB23" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -2739,7 +2739,7 @@
       <c r="AA24" s="3" t="n"/>
       <c r="AB24" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2833,7 @@
       <c r="AA25" s="3" t="n"/>
       <c r="AB25" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -2927,7 +2927,7 @@
       <c r="AA26" s="3" t="n"/>
       <c r="AB26" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -3025,7 +3025,7 @@
       <c r="AA27" s="3" t="n"/>
       <c r="AB27" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -3123,7 +3123,7 @@
       <c r="AA28" s="3" t="n"/>
       <c r="AB28" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -3221,7 +3221,7 @@
       <c r="AA29" s="3" t="n"/>
       <c r="AB29" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -3319,7 +3319,7 @@
       <c r="AA30" s="3" t="n"/>
       <c r="AB30" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -3417,7 +3417,7 @@
       <c r="AA31" s="3" t="n"/>
       <c r="AB31" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -3511,7 +3511,7 @@
       <c r="AA32" s="3" t="n"/>
       <c r="AB32" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -3609,7 +3609,7 @@
       <c r="AA33" s="3" t="n"/>
       <c r="AB33" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -3703,7 +3703,7 @@
       <c r="AA34" s="3" t="n"/>
       <c r="AB34" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -3789,7 +3789,7 @@
       <c r="AA35" s="3" t="n"/>
       <c r="AB35" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -3887,7 +3887,7 @@
       <c r="AA36" s="3" t="n"/>
       <c r="AB36" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -3981,7 +3981,7 @@
       <c r="AA37" s="3" t="n"/>
       <c r="AB37" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -4079,7 +4079,7 @@
       <c r="AA38" s="3" t="n"/>
       <c r="AB38" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -4173,7 +4173,7 @@
       <c r="AA39" s="3" t="n"/>
       <c r="AB39" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -4271,7 +4271,7 @@
       <c r="AA40" s="3" t="n"/>
       <c r="AB40" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -4365,7 +4365,7 @@
       <c r="AA41" s="3" t="n"/>
       <c r="AB41" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -4463,7 +4463,7 @@
       <c r="AA42" s="3" t="n"/>
       <c r="AB42" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -4561,7 +4561,7 @@
       <c r="AA43" s="3" t="n"/>
       <c r="AB43" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -4655,7 +4655,7 @@
       <c r="AA44" s="3" t="n"/>
       <c r="AB44" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -4753,7 +4753,7 @@
       <c r="AA45" s="3" t="n"/>
       <c r="AB45" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -4843,7 +4843,7 @@
       <c r="AA46" s="3" t="n"/>
       <c r="AB46" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -4941,7 +4941,7 @@
       <c r="AA47" s="3" t="n"/>
       <c r="AB47" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -5039,7 +5039,7 @@
       <c r="AA48" s="3" t="n"/>
       <c r="AB48" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -5125,7 +5125,7 @@
       <c r="AA49" s="3" t="n"/>
       <c r="AB49" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -5219,7 +5219,7 @@
       <c r="AA50" s="3" t="n"/>
       <c r="AB50" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -5317,7 +5317,7 @@
       <c r="AA51" s="3" t="n"/>
       <c r="AB51" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -5407,7 +5407,7 @@
       <c r="AA52" s="3" t="n"/>
       <c r="AB52" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -5505,7 +5505,7 @@
       <c r="AA53" s="3" t="n"/>
       <c r="AB53" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       <c r="AA54" s="3" t="n"/>
       <c r="AB54" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -5693,7 +5693,7 @@
       <c r="AA55" s="3" t="n"/>
       <c r="AB55" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -5783,7 +5783,7 @@
       <c r="AA56" s="3" t="n"/>
       <c r="AB56" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -5877,7 +5877,7 @@
       <c r="AA57" s="3" t="n"/>
       <c r="AB57" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -5975,7 +5975,7 @@
       <c r="AA58" s="3" t="n"/>
       <c r="AB58" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6069,7 +6069,7 @@
       <c r="AA59" s="3" t="n"/>
       <c r="AB59" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6167,7 +6167,7 @@
       <c r="AA60" s="3" t="n"/>
       <c r="AB60" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6261,7 +6261,7 @@
       <c r="AA61" s="3" t="n"/>
       <c r="AB61" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6347,7 +6347,7 @@
       <c r="AA62" s="3" t="n"/>
       <c r="AB62" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6437,7 +6437,7 @@
       <c r="AA63" s="3" t="n"/>
       <c r="AB63" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6535,7 +6535,7 @@
       <c r="AA64" s="3" t="n"/>
       <c r="AB64" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6633,7 +6633,7 @@
       <c r="AA65" s="3" t="n"/>
       <c r="AB65" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6731,7 +6731,7 @@
       <c r="AA66" s="3" t="n"/>
       <c r="AB66" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6825,7 +6825,7 @@
       <c r="AA67" s="3" t="n"/>
       <c r="AB67" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6923,7 +6923,7 @@
       <c r="AA68" s="3" t="n"/>
       <c r="AB68" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -7021,7 +7021,7 @@
       <c r="AA69" s="3" t="n"/>
       <c r="AB69" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -7119,7 +7119,7 @@
       <c r="AA70" s="3" t="n"/>
       <c r="AB70" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -7217,7 +7217,7 @@
       <c r="AA71" s="3" t="n"/>
       <c r="AB71" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -7303,7 +7303,7 @@
       <c r="AA72" s="3" t="n"/>
       <c r="AB72" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       <c r="AA73" s="3" t="n"/>
       <c r="AB73" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -7483,7 +7483,7 @@
       <c r="AA74" s="3" t="n"/>
       <c r="AB74" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -7585,7 +7585,7 @@
       <c r="AA75" s="3" t="n"/>
       <c r="AB75" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -7675,7 +7675,7 @@
       <c r="AA76" s="3" t="n"/>
       <c r="AB76" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -7765,7 +7765,7 @@
       <c r="AA77" s="3" t="n"/>
       <c r="AB77" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -7859,7 +7859,7 @@
       <c r="AA78" s="3" t="n"/>
       <c r="AB78" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -7961,7 +7961,7 @@
       <c r="AA79" s="3" t="n"/>
       <c r="AB79" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -8051,7 +8051,7 @@
       <c r="AA80" s="3" t="n"/>
       <c r="AB80" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -8145,7 +8145,7 @@
       <c r="AA81" s="3" t="n"/>
       <c r="AB81" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -8239,7 +8239,7 @@
       <c r="AA82" s="3" t="n"/>
       <c r="AB82" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -8337,7 +8337,7 @@
       <c r="AA83" s="3" t="n"/>
       <c r="AB83" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -8435,7 +8435,7 @@
       <c r="AA84" s="3" t="n"/>
       <c r="AB84" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -8529,7 +8529,7 @@
       <c r="AA85" s="3" t="n"/>
       <c r="AB85" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -8619,7 +8619,7 @@
       <c r="AA86" s="3" t="n"/>
       <c r="AB86" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -8721,7 +8721,7 @@
       <c r="AA87" s="3" t="n"/>
       <c r="AB87" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -8819,7 +8819,7 @@
       <c r="AA88" s="3" t="n"/>
       <c r="AB88" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -8905,7 +8905,7 @@
       <c r="AA89" s="3" t="n"/>
       <c r="AB89" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -8999,7 +8999,7 @@
       <c r="AA90" s="3" t="n"/>
       <c r="AB90" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -9097,7 +9097,7 @@
       <c r="AA91" s="3" t="n"/>
       <c r="AB91" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -9195,7 +9195,7 @@
       <c r="AA92" s="3" t="n"/>
       <c r="AB92" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -9293,7 +9293,7 @@
       <c r="AA93" s="3" t="n"/>
       <c r="AB93" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -9383,7 +9383,7 @@
       <c r="AA94" s="3" t="n"/>
       <c r="AB94" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -9477,7 +9477,7 @@
       <c r="AA95" s="3" t="n"/>
       <c r="AB95" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -9575,7 +9575,7 @@
       <c r="AA96" s="3" t="n"/>
       <c r="AB96" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -9673,7 +9673,7 @@
       <c r="AA97" s="3" t="n"/>
       <c r="AB97" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -9767,7 +9767,7 @@
       <c r="AA98" s="3" t="n"/>
       <c r="AB98" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -9865,7 +9865,7 @@
       <c r="AA99" s="3" t="n"/>
       <c r="AB99" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -9963,7 +9963,7 @@
       <c r="AA100" s="3" t="n"/>
       <c r="AB100" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -10061,7 +10061,7 @@
       <c r="AA101" s="3" t="n"/>
       <c r="AB101" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -10151,7 +10151,7 @@
       <c r="AA102" s="3" t="n"/>
       <c r="AB102" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -10249,7 +10249,7 @@
       <c r="AA103" s="3" t="n"/>
       <c r="AB103" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -10347,7 +10347,7 @@
       <c r="AA104" s="3" t="n"/>
       <c r="AB104" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -10449,7 +10449,7 @@
       <c r="AA105" s="3" t="n"/>
       <c r="AB105" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -10543,7 +10543,7 @@
       <c r="AA106" s="3" t="n"/>
       <c r="AB106" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -10645,7 +10645,7 @@
       <c r="AA107" s="3" t="n"/>
       <c r="AB107" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -10739,7 +10739,7 @@
       <c r="AA108" s="3" t="n"/>
       <c r="AB108" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -10833,7 +10833,7 @@
       <c r="AA109" s="3" t="n"/>
       <c r="AB109" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -10935,7 +10935,7 @@
       <c r="AA110" s="3" t="n"/>
       <c r="AB110" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -11037,7 +11037,7 @@
       <c r="AA111" s="3" t="n"/>
       <c r="AB111" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -11135,7 +11135,7 @@
       <c r="AA112" s="3" t="n"/>
       <c r="AB112" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -11225,7 +11225,7 @@
       <c r="AA113" s="3" t="n"/>
       <c r="AB113" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -11323,7 +11323,7 @@
       <c r="AA114" s="3" t="n"/>
       <c r="AB114" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -11413,7 +11413,7 @@
       <c r="AA115" s="3" t="n"/>
       <c r="AB115" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -11511,7 +11511,7 @@
       <c r="AA116" s="3" t="n"/>
       <c r="AB116" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -11609,7 +11609,7 @@
       <c r="AA117" s="3" t="n"/>
       <c r="AB117" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -11707,7 +11707,7 @@
       <c r="AA118" s="3" t="n"/>
       <c r="AB118" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -11805,7 +11805,7 @@
       <c r="AA119" s="3" t="n"/>
       <c r="AB119" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -11903,7 +11903,7 @@
       <c r="AA120" s="3" t="n"/>
       <c r="AB120" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -11993,7 +11993,7 @@
       <c r="AA121" s="3" t="n"/>
       <c r="AB121" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -12091,7 +12091,7 @@
       <c r="AA122" s="3" t="n"/>
       <c r="AB122" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -12189,7 +12189,7 @@
       <c r="AA123" s="3" t="n"/>
       <c r="AB123" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -12283,7 +12283,7 @@
       <c r="AA124" s="3" t="n"/>
       <c r="AB124" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -12377,7 +12377,7 @@
       <c r="AA125" s="3" t="n"/>
       <c r="AB125" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -12467,7 +12467,7 @@
       <c r="AA126" s="3" t="n"/>
       <c r="AB126" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -12561,7 +12561,7 @@
       <c r="AA127" s="3" t="n"/>
       <c r="AB127" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -12659,7 +12659,7 @@
       <c r="AA128" s="3" t="n"/>
       <c r="AB128" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -12757,7 +12757,7 @@
       <c r="AA129" s="3" t="n"/>
       <c r="AB129" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -12855,7 +12855,7 @@
       <c r="AA130" s="3" t="n"/>
       <c r="AB130" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -12953,7 +12953,7 @@
       <c r="AA131" s="3" t="n"/>
       <c r="AB131" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -13043,7 +13043,7 @@
       <c r="AA132" s="3" t="n"/>
       <c r="AB132" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -13141,7 +13141,7 @@
       <c r="AA133" s="3" t="n"/>
       <c r="AB133" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -13235,7 +13235,7 @@
       <c r="AA134" s="3" t="n"/>
       <c r="AB134" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -13333,7 +13333,7 @@
       <c r="AA135" s="3" t="n"/>
       <c r="AB135" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -13427,7 +13427,7 @@
       <c r="AA136" s="3" t="n"/>
       <c r="AB136" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -13525,7 +13525,7 @@
       <c r="AA137" s="3" t="n"/>
       <c r="AB137" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -13619,7 +13619,7 @@
       <c r="AA138" s="3" t="n"/>
       <c r="AB138" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -13713,7 +13713,7 @@
       <c r="AA139" s="3" t="n"/>
       <c r="AB139" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -13811,7 +13811,7 @@
       <c r="AA140" s="3" t="n"/>
       <c r="AB140" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -13905,7 +13905,7 @@
       <c r="AA141" s="3" t="n"/>
       <c r="AB141" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -13999,7 +13999,7 @@
       <c r="AA142" s="3" t="n"/>
       <c r="AB142" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -14089,7 +14089,7 @@
       <c r="AA143" s="3" t="n"/>
       <c r="AB143" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -14183,7 +14183,7 @@
       <c r="AA144" s="3" t="n"/>
       <c r="AB144" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh the corpus after fetching 22 open full texts; add the review-before-commit note
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/corpus/corpus.xlsx
+++ b/corpus/corpus.xlsx
@@ -677,15 +677,15 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr"/>
-      <c r="Q2" s="3" t="inlineStr"/>
-      <c r="R2" s="3" t="inlineStr"/>
-      <c r="S2" s="3" t="inlineStr"/>
-      <c r="T2" s="3" t="inlineStr"/>
-      <c r="U2" s="3" t="inlineStr"/>
-      <c r="V2" s="3" t="inlineStr"/>
-      <c r="W2" s="3" t="inlineStr"/>
-      <c r="X2" s="3" t="inlineStr"/>
+      <c r="P2" s="3" t="n"/>
+      <c r="Q2" s="3" t="n"/>
+      <c r="R2" s="3" t="n"/>
+      <c r="S2" s="3" t="n"/>
+      <c r="T2" s="3" t="n"/>
+      <c r="U2" s="3" t="n"/>
+      <c r="V2" s="3" t="n"/>
+      <c r="W2" s="3" t="n"/>
+      <c r="X2" s="3" t="n"/>
       <c r="Y2" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -696,7 +696,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA2" s="3" t="inlineStr"/>
+      <c r="AA2" s="3" t="n"/>
       <c r="AB2" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -857,15 +857,15 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr"/>
-      <c r="Q4" s="3" t="inlineStr"/>
-      <c r="R4" s="3" t="inlineStr"/>
-      <c r="S4" s="3" t="inlineStr"/>
-      <c r="T4" s="3" t="inlineStr"/>
-      <c r="U4" s="3" t="inlineStr"/>
-      <c r="V4" s="3" t="inlineStr"/>
-      <c r="W4" s="3" t="inlineStr"/>
-      <c r="X4" s="3" t="inlineStr"/>
+      <c r="P4" s="3" t="n"/>
+      <c r="Q4" s="3" t="n"/>
+      <c r="R4" s="3" t="n"/>
+      <c r="S4" s="3" t="n"/>
+      <c r="T4" s="3" t="n"/>
+      <c r="U4" s="3" t="n"/>
+      <c r="V4" s="3" t="n"/>
+      <c r="W4" s="3" t="n"/>
+      <c r="X4" s="3" t="n"/>
       <c r="Y4" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -876,7 +876,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA4" s="3" t="inlineStr"/>
+      <c r="AA4" s="3" t="n"/>
       <c r="AB4" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -2627,18 +2627,18 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P23" s="3" t="inlineStr"/>
-      <c r="Q23" s="3" t="inlineStr"/>
-      <c r="R23" s="3" t="inlineStr"/>
-      <c r="S23" s="3" t="inlineStr"/>
-      <c r="T23" s="3" t="inlineStr"/>
-      <c r="U23" s="3" t="inlineStr"/>
-      <c r="V23" s="3" t="inlineStr"/>
-      <c r="W23" s="3" t="inlineStr"/>
-      <c r="X23" s="3" t="inlineStr"/>
+      <c r="P23" s="3" t="n"/>
+      <c r="Q23" s="3" t="n"/>
+      <c r="R23" s="3" t="n"/>
+      <c r="S23" s="3" t="n"/>
+      <c r="T23" s="3" t="n"/>
+      <c r="U23" s="3" t="n"/>
+      <c r="V23" s="3" t="n"/>
+      <c r="W23" s="3" t="n"/>
+      <c r="X23" s="3" t="n"/>
       <c r="Y23" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z23" s="3" t="inlineStr">
@@ -2646,7 +2646,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA23" s="3" t="inlineStr"/>
+      <c r="AA23" s="3" t="n"/>
       <c r="AB23" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -2717,15 +2717,15 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P24" s="3" t="inlineStr"/>
-      <c r="Q24" s="3" t="inlineStr"/>
-      <c r="R24" s="3" t="inlineStr"/>
-      <c r="S24" s="3" t="inlineStr"/>
-      <c r="T24" s="3" t="inlineStr"/>
-      <c r="U24" s="3" t="inlineStr"/>
-      <c r="V24" s="3" t="inlineStr"/>
-      <c r="W24" s="3" t="inlineStr"/>
-      <c r="X24" s="3" t="inlineStr"/>
+      <c r="P24" s="3" t="n"/>
+      <c r="Q24" s="3" t="n"/>
+      <c r="R24" s="3" t="n"/>
+      <c r="S24" s="3" t="n"/>
+      <c r="T24" s="3" t="n"/>
+      <c r="U24" s="3" t="n"/>
+      <c r="V24" s="3" t="n"/>
+      <c r="W24" s="3" t="n"/>
+      <c r="X24" s="3" t="n"/>
       <c r="Y24" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -2736,7 +2736,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA24" s="3" t="inlineStr"/>
+      <c r="AA24" s="3" t="n"/>
       <c r="AB24" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -2811,18 +2811,18 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P25" s="3" t="inlineStr"/>
-      <c r="Q25" s="3" t="inlineStr"/>
-      <c r="R25" s="3" t="inlineStr"/>
-      <c r="S25" s="3" t="inlineStr"/>
-      <c r="T25" s="3" t="inlineStr"/>
-      <c r="U25" s="3" t="inlineStr"/>
-      <c r="V25" s="3" t="inlineStr"/>
-      <c r="W25" s="3" t="inlineStr"/>
-      <c r="X25" s="3" t="inlineStr"/>
+      <c r="P25" s="3" t="n"/>
+      <c r="Q25" s="3" t="n"/>
+      <c r="R25" s="3" t="n"/>
+      <c r="S25" s="3" t="n"/>
+      <c r="T25" s="3" t="n"/>
+      <c r="U25" s="3" t="n"/>
+      <c r="V25" s="3" t="n"/>
+      <c r="W25" s="3" t="n"/>
+      <c r="X25" s="3" t="n"/>
       <c r="Y25" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z25" s="3" t="inlineStr">
@@ -2830,7 +2830,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA25" s="3" t="inlineStr"/>
+      <c r="AA25" s="3" t="n"/>
       <c r="AB25" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -3003,18 +3003,18 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P27" s="3" t="inlineStr"/>
-      <c r="Q27" s="3" t="inlineStr"/>
-      <c r="R27" s="3" t="inlineStr"/>
-      <c r="S27" s="3" t="inlineStr"/>
-      <c r="T27" s="3" t="inlineStr"/>
-      <c r="U27" s="3" t="inlineStr"/>
-      <c r="V27" s="3" t="inlineStr"/>
-      <c r="W27" s="3" t="inlineStr"/>
-      <c r="X27" s="3" t="inlineStr"/>
+      <c r="P27" s="3" t="n"/>
+      <c r="Q27" s="3" t="n"/>
+      <c r="R27" s="3" t="n"/>
+      <c r="S27" s="3" t="n"/>
+      <c r="T27" s="3" t="n"/>
+      <c r="U27" s="3" t="n"/>
+      <c r="V27" s="3" t="n"/>
+      <c r="W27" s="3" t="n"/>
+      <c r="X27" s="3" t="n"/>
       <c r="Y27" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z27" s="3" t="inlineStr">
@@ -3022,7 +3022,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA27" s="3" t="inlineStr"/>
+      <c r="AA27" s="3" t="n"/>
       <c r="AB27" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -3097,22 +3097,22 @@
           <t>full text</t>
         </is>
       </c>
-      <c r="P28" s="3" t="inlineStr"/>
-      <c r="Q28" s="3" t="inlineStr"/>
-      <c r="R28" s="3" t="inlineStr"/>
-      <c r="S28" s="3" t="inlineStr"/>
-      <c r="T28" s="3" t="inlineStr"/>
-      <c r="U28" s="3" t="inlineStr"/>
-      <c r="V28" s="3" t="inlineStr"/>
-      <c r="W28" s="3" t="inlineStr"/>
-      <c r="X28" s="3" t="inlineStr"/>
+      <c r="P28" s="3" t="n"/>
+      <c r="Q28" s="3" t="n"/>
+      <c r="R28" s="3" t="n"/>
+      <c r="S28" s="3" t="n"/>
+      <c r="T28" s="3" t="n"/>
+      <c r="U28" s="3" t="n"/>
+      <c r="V28" s="3" t="n"/>
+      <c r="W28" s="3" t="n"/>
+      <c r="X28" s="3" t="n"/>
       <c r="Y28" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z28" s="3" t="inlineStr"/>
-      <c r="AA28" s="3" t="inlineStr"/>
+      <c r="AA28" s="3" t="n"/>
       <c r="AB28" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -3187,22 +3187,22 @@
           <t>full text</t>
         </is>
       </c>
-      <c r="P29" s="3" t="inlineStr"/>
-      <c r="Q29" s="3" t="inlineStr"/>
-      <c r="R29" s="3" t="inlineStr"/>
-      <c r="S29" s="3" t="inlineStr"/>
-      <c r="T29" s="3" t="inlineStr"/>
-      <c r="U29" s="3" t="inlineStr"/>
-      <c r="V29" s="3" t="inlineStr"/>
-      <c r="W29" s="3" t="inlineStr"/>
-      <c r="X29" s="3" t="inlineStr"/>
+      <c r="P29" s="3" t="n"/>
+      <c r="Q29" s="3" t="n"/>
+      <c r="R29" s="3" t="n"/>
+      <c r="S29" s="3" t="n"/>
+      <c r="T29" s="3" t="n"/>
+      <c r="U29" s="3" t="n"/>
+      <c r="V29" s="3" t="n"/>
+      <c r="W29" s="3" t="n"/>
+      <c r="X29" s="3" t="n"/>
       <c r="Y29" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z29" s="3" t="inlineStr"/>
-      <c r="AA29" s="3" t="inlineStr"/>
+      <c r="AA29" s="3" t="n"/>
       <c r="AB29" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -3461,15 +3461,15 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P32" s="3" t="inlineStr"/>
-      <c r="Q32" s="3" t="inlineStr"/>
-      <c r="R32" s="3" t="inlineStr"/>
-      <c r="S32" s="3" t="inlineStr"/>
-      <c r="T32" s="3" t="inlineStr"/>
-      <c r="U32" s="3" t="inlineStr"/>
-      <c r="V32" s="3" t="inlineStr"/>
-      <c r="W32" s="3" t="inlineStr"/>
-      <c r="X32" s="3" t="inlineStr"/>
+      <c r="P32" s="3" t="n"/>
+      <c r="Q32" s="3" t="n"/>
+      <c r="R32" s="3" t="n"/>
+      <c r="S32" s="3" t="n"/>
+      <c r="T32" s="3" t="n"/>
+      <c r="U32" s="3" t="n"/>
+      <c r="V32" s="3" t="n"/>
+      <c r="W32" s="3" t="n"/>
+      <c r="X32" s="3" t="n"/>
       <c r="Y32" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -3480,7 +3480,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA32" s="3" t="inlineStr"/>
+      <c r="AA32" s="3" t="n"/>
       <c r="AB32" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -3645,15 +3645,15 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P34" s="3" t="inlineStr"/>
-      <c r="Q34" s="3" t="inlineStr"/>
-      <c r="R34" s="3" t="inlineStr"/>
-      <c r="S34" s="3" t="inlineStr"/>
-      <c r="T34" s="3" t="inlineStr"/>
-      <c r="U34" s="3" t="inlineStr"/>
-      <c r="V34" s="3" t="inlineStr"/>
-      <c r="W34" s="3" t="inlineStr"/>
-      <c r="X34" s="3" t="inlineStr"/>
+      <c r="P34" s="3" t="n"/>
+      <c r="Q34" s="3" t="n"/>
+      <c r="R34" s="3" t="n"/>
+      <c r="S34" s="3" t="n"/>
+      <c r="T34" s="3" t="n"/>
+      <c r="U34" s="3" t="n"/>
+      <c r="V34" s="3" t="n"/>
+      <c r="W34" s="3" t="n"/>
+      <c r="X34" s="3" t="n"/>
       <c r="Y34" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -3664,7 +3664,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA34" s="3" t="inlineStr"/>
+      <c r="AA34" s="3" t="n"/>
       <c r="AB34" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -3833,22 +3833,22 @@
           <t>full text</t>
         </is>
       </c>
-      <c r="P36" s="3" t="inlineStr"/>
-      <c r="Q36" s="3" t="inlineStr"/>
-      <c r="R36" s="3" t="inlineStr"/>
-      <c r="S36" s="3" t="inlineStr"/>
-      <c r="T36" s="3" t="inlineStr"/>
-      <c r="U36" s="3" t="inlineStr"/>
-      <c r="V36" s="3" t="inlineStr"/>
-      <c r="W36" s="3" t="inlineStr"/>
-      <c r="X36" s="3" t="inlineStr"/>
+      <c r="P36" s="3" t="n"/>
+      <c r="Q36" s="3" t="n"/>
+      <c r="R36" s="3" t="n"/>
+      <c r="S36" s="3" t="n"/>
+      <c r="T36" s="3" t="n"/>
+      <c r="U36" s="3" t="n"/>
+      <c r="V36" s="3" t="n"/>
+      <c r="W36" s="3" t="n"/>
+      <c r="X36" s="3" t="n"/>
       <c r="Y36" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z36" s="3" t="inlineStr"/>
-      <c r="AA36" s="3" t="inlineStr"/>
+      <c r="AA36" s="3" t="n"/>
       <c r="AB36" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -4209,15 +4209,15 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P40" s="3" t="inlineStr"/>
-      <c r="Q40" s="3" t="inlineStr"/>
-      <c r="R40" s="3" t="inlineStr"/>
-      <c r="S40" s="3" t="inlineStr"/>
-      <c r="T40" s="3" t="inlineStr"/>
-      <c r="U40" s="3" t="inlineStr"/>
-      <c r="V40" s="3" t="inlineStr"/>
-      <c r="W40" s="3" t="inlineStr"/>
-      <c r="X40" s="3" t="inlineStr"/>
+      <c r="P40" s="3" t="n"/>
+      <c r="Q40" s="3" t="n"/>
+      <c r="R40" s="3" t="n"/>
+      <c r="S40" s="3" t="n"/>
+      <c r="T40" s="3" t="n"/>
+      <c r="U40" s="3" t="n"/>
+      <c r="V40" s="3" t="n"/>
+      <c r="W40" s="3" t="n"/>
+      <c r="X40" s="3" t="n"/>
       <c r="Y40" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -4228,7 +4228,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA40" s="3" t="inlineStr"/>
+      <c r="AA40" s="3" t="n"/>
       <c r="AB40" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -4299,15 +4299,15 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P41" s="3" t="inlineStr"/>
-      <c r="Q41" s="3" t="inlineStr"/>
-      <c r="R41" s="3" t="inlineStr"/>
-      <c r="S41" s="3" t="inlineStr"/>
-      <c r="T41" s="3" t="inlineStr"/>
-      <c r="U41" s="3" t="inlineStr"/>
-      <c r="V41" s="3" t="inlineStr"/>
-      <c r="W41" s="3" t="inlineStr"/>
-      <c r="X41" s="3" t="inlineStr"/>
+      <c r="P41" s="3" t="n"/>
+      <c r="Q41" s="3" t="n"/>
+      <c r="R41" s="3" t="n"/>
+      <c r="S41" s="3" t="n"/>
+      <c r="T41" s="3" t="n"/>
+      <c r="U41" s="3" t="n"/>
+      <c r="V41" s="3" t="n"/>
+      <c r="W41" s="3" t="n"/>
+      <c r="X41" s="3" t="n"/>
       <c r="Y41" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -4318,7 +4318,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA41" s="3" t="inlineStr"/>
+      <c r="AA41" s="3" t="n"/>
       <c r="AB41" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -4683,15 +4683,15 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P45" s="3" t="inlineStr"/>
-      <c r="Q45" s="3" t="inlineStr"/>
-      <c r="R45" s="3" t="inlineStr"/>
-      <c r="S45" s="3" t="inlineStr"/>
-      <c r="T45" s="3" t="inlineStr"/>
-      <c r="U45" s="3" t="inlineStr"/>
-      <c r="V45" s="3" t="inlineStr"/>
-      <c r="W45" s="3" t="inlineStr"/>
-      <c r="X45" s="3" t="inlineStr"/>
+      <c r="P45" s="3" t="n"/>
+      <c r="Q45" s="3" t="n"/>
+      <c r="R45" s="3" t="n"/>
+      <c r="S45" s="3" t="n"/>
+      <c r="T45" s="3" t="n"/>
+      <c r="U45" s="3" t="n"/>
+      <c r="V45" s="3" t="n"/>
+      <c r="W45" s="3" t="n"/>
+      <c r="X45" s="3" t="n"/>
       <c r="Y45" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -4702,7 +4702,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA45" s="3" t="inlineStr"/>
+      <c r="AA45" s="3" t="n"/>
       <c r="AB45" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -4871,15 +4871,15 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P47" s="3" t="inlineStr"/>
-      <c r="Q47" s="3" t="inlineStr"/>
-      <c r="R47" s="3" t="inlineStr"/>
-      <c r="S47" s="3" t="inlineStr"/>
-      <c r="T47" s="3" t="inlineStr"/>
-      <c r="U47" s="3" t="inlineStr"/>
-      <c r="V47" s="3" t="inlineStr"/>
-      <c r="W47" s="3" t="inlineStr"/>
-      <c r="X47" s="3" t="inlineStr"/>
+      <c r="P47" s="3" t="n"/>
+      <c r="Q47" s="3" t="n"/>
+      <c r="R47" s="3" t="n"/>
+      <c r="S47" s="3" t="n"/>
+      <c r="T47" s="3" t="n"/>
+      <c r="U47" s="3" t="n"/>
+      <c r="V47" s="3" t="n"/>
+      <c r="W47" s="3" t="n"/>
+      <c r="X47" s="3" t="n"/>
       <c r="Y47" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -4890,7 +4890,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA47" s="3" t="inlineStr"/>
+      <c r="AA47" s="3" t="n"/>
       <c r="AB47" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -5533,18 +5533,18 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P54" s="3" t="inlineStr"/>
-      <c r="Q54" s="3" t="inlineStr"/>
-      <c r="R54" s="3" t="inlineStr"/>
-      <c r="S54" s="3" t="inlineStr"/>
-      <c r="T54" s="3" t="inlineStr"/>
-      <c r="U54" s="3" t="inlineStr"/>
-      <c r="V54" s="3" t="inlineStr"/>
-      <c r="W54" s="3" t="inlineStr"/>
-      <c r="X54" s="3" t="inlineStr"/>
+      <c r="P54" s="3" t="n"/>
+      <c r="Q54" s="3" t="n"/>
+      <c r="R54" s="3" t="n"/>
+      <c r="S54" s="3" t="n"/>
+      <c r="T54" s="3" t="n"/>
+      <c r="U54" s="3" t="n"/>
+      <c r="V54" s="3" t="n"/>
+      <c r="W54" s="3" t="n"/>
+      <c r="X54" s="3" t="n"/>
       <c r="Y54" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z54" s="3" t="inlineStr">
@@ -5552,7 +5552,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA54" s="3" t="inlineStr"/>
+      <c r="AA54" s="3" t="n"/>
       <c r="AB54" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -5913,18 +5913,18 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P58" s="3" t="inlineStr"/>
-      <c r="Q58" s="3" t="inlineStr"/>
-      <c r="R58" s="3" t="inlineStr"/>
-      <c r="S58" s="3" t="inlineStr"/>
-      <c r="T58" s="3" t="inlineStr"/>
-      <c r="U58" s="3" t="inlineStr"/>
-      <c r="V58" s="3" t="inlineStr"/>
-      <c r="W58" s="3" t="inlineStr"/>
-      <c r="X58" s="3" t="inlineStr"/>
+      <c r="P58" s="3" t="n"/>
+      <c r="Q58" s="3" t="n"/>
+      <c r="R58" s="3" t="n"/>
+      <c r="S58" s="3" t="n"/>
+      <c r="T58" s="3" t="n"/>
+      <c r="U58" s="3" t="n"/>
+      <c r="V58" s="3" t="n"/>
+      <c r="W58" s="3" t="n"/>
+      <c r="X58" s="3" t="n"/>
       <c r="Y58" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z58" s="3" t="inlineStr">
@@ -5932,7 +5932,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA58" s="3" t="inlineStr"/>
+      <c r="AA58" s="3" t="n"/>
       <c r="AB58" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -6199,15 +6199,15 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P61" s="3" t="inlineStr"/>
-      <c r="Q61" s="3" t="inlineStr"/>
-      <c r="R61" s="3" t="inlineStr"/>
-      <c r="S61" s="3" t="inlineStr"/>
-      <c r="T61" s="3" t="inlineStr"/>
-      <c r="U61" s="3" t="inlineStr"/>
-      <c r="V61" s="3" t="inlineStr"/>
-      <c r="W61" s="3" t="inlineStr"/>
-      <c r="X61" s="3" t="inlineStr"/>
+      <c r="P61" s="3" t="n"/>
+      <c r="Q61" s="3" t="n"/>
+      <c r="R61" s="3" t="n"/>
+      <c r="S61" s="3" t="n"/>
+      <c r="T61" s="3" t="n"/>
+      <c r="U61" s="3" t="n"/>
+      <c r="V61" s="3" t="n"/>
+      <c r="W61" s="3" t="n"/>
+      <c r="X61" s="3" t="n"/>
       <c r="Y61" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -6218,7 +6218,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA61" s="3" t="inlineStr"/>
+      <c r="AA61" s="3" t="n"/>
       <c r="AB61" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -6771,18 +6771,18 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P67" s="3" t="inlineStr"/>
-      <c r="Q67" s="3" t="inlineStr"/>
-      <c r="R67" s="3" t="inlineStr"/>
-      <c r="S67" s="3" t="inlineStr"/>
-      <c r="T67" s="3" t="inlineStr"/>
-      <c r="U67" s="3" t="inlineStr"/>
-      <c r="V67" s="3" t="inlineStr"/>
-      <c r="W67" s="3" t="inlineStr"/>
-      <c r="X67" s="3" t="inlineStr"/>
+      <c r="P67" s="3" t="n"/>
+      <c r="Q67" s="3" t="n"/>
+      <c r="R67" s="3" t="n"/>
+      <c r="S67" s="3" t="n"/>
+      <c r="T67" s="3" t="n"/>
+      <c r="U67" s="3" t="n"/>
+      <c r="V67" s="3" t="n"/>
+      <c r="W67" s="3" t="n"/>
+      <c r="X67" s="3" t="n"/>
       <c r="Y67" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z67" s="3" t="inlineStr">
@@ -6790,7 +6790,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA67" s="3" t="inlineStr"/>
+      <c r="AA67" s="3" t="n"/>
       <c r="AB67" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -7041,15 +7041,15 @@
           <t>abstract, full text</t>
         </is>
       </c>
-      <c r="P70" s="3" t="inlineStr"/>
-      <c r="Q70" s="3" t="inlineStr"/>
-      <c r="R70" s="3" t="inlineStr"/>
-      <c r="S70" s="3" t="inlineStr"/>
-      <c r="T70" s="3" t="inlineStr"/>
-      <c r="U70" s="3" t="inlineStr"/>
-      <c r="V70" s="3" t="inlineStr"/>
-      <c r="W70" s="3" t="inlineStr"/>
-      <c r="X70" s="3" t="inlineStr"/>
+      <c r="P70" s="3" t="n"/>
+      <c r="Q70" s="3" t="n"/>
+      <c r="R70" s="3" t="n"/>
+      <c r="S70" s="3" t="n"/>
+      <c r="T70" s="3" t="n"/>
+      <c r="U70" s="3" t="n"/>
+      <c r="V70" s="3" t="n"/>
+      <c r="W70" s="3" t="n"/>
+      <c r="X70" s="3" t="n"/>
       <c r="Y70" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -7060,7 +7060,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA70" s="3" t="inlineStr"/>
+      <c r="AA70" s="3" t="n"/>
       <c r="AB70" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -7421,18 +7421,18 @@
           <t>abstract, full text</t>
         </is>
       </c>
-      <c r="P74" s="3" t="inlineStr"/>
-      <c r="Q74" s="3" t="inlineStr"/>
-      <c r="R74" s="3" t="inlineStr"/>
-      <c r="S74" s="3" t="inlineStr"/>
-      <c r="T74" s="3" t="inlineStr"/>
-      <c r="U74" s="3" t="inlineStr"/>
-      <c r="V74" s="3" t="inlineStr"/>
-      <c r="W74" s="3" t="inlineStr"/>
-      <c r="X74" s="3" t="inlineStr"/>
+      <c r="P74" s="3" t="n"/>
+      <c r="Q74" s="3" t="n"/>
+      <c r="R74" s="3" t="n"/>
+      <c r="S74" s="3" t="n"/>
+      <c r="T74" s="3" t="n"/>
+      <c r="U74" s="3" t="n"/>
+      <c r="V74" s="3" t="n"/>
+      <c r="W74" s="3" t="n"/>
+      <c r="X74" s="3" t="n"/>
       <c r="Y74" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z74" s="3" t="inlineStr">
@@ -7440,7 +7440,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA74" s="3" t="inlineStr"/>
+      <c r="AA74" s="3" t="n"/>
       <c r="AB74" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -7609,18 +7609,18 @@
           <t>abstract, full text</t>
         </is>
       </c>
-      <c r="P76" s="3" t="inlineStr"/>
-      <c r="Q76" s="3" t="inlineStr"/>
-      <c r="R76" s="3" t="inlineStr"/>
-      <c r="S76" s="3" t="inlineStr"/>
-      <c r="T76" s="3" t="inlineStr"/>
-      <c r="U76" s="3" t="inlineStr"/>
-      <c r="V76" s="3" t="inlineStr"/>
-      <c r="W76" s="3" t="inlineStr"/>
-      <c r="X76" s="3" t="inlineStr"/>
+      <c r="P76" s="3" t="n"/>
+      <c r="Q76" s="3" t="n"/>
+      <c r="R76" s="3" t="n"/>
+      <c r="S76" s="3" t="n"/>
+      <c r="T76" s="3" t="n"/>
+      <c r="U76" s="3" t="n"/>
+      <c r="V76" s="3" t="n"/>
+      <c r="W76" s="3" t="n"/>
+      <c r="X76" s="3" t="n"/>
       <c r="Y76" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z76" s="3" t="inlineStr">
@@ -7628,7 +7628,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA76" s="3" t="inlineStr"/>
+      <c r="AA76" s="3" t="n"/>
       <c r="AB76" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -7801,15 +7801,15 @@
           <t>abstract, full text, recall</t>
         </is>
       </c>
-      <c r="P78" s="3" t="inlineStr"/>
-      <c r="Q78" s="3" t="inlineStr"/>
-      <c r="R78" s="3" t="inlineStr"/>
-      <c r="S78" s="3" t="inlineStr"/>
-      <c r="T78" s="3" t="inlineStr"/>
-      <c r="U78" s="3" t="inlineStr"/>
-      <c r="V78" s="3" t="inlineStr"/>
-      <c r="W78" s="3" t="inlineStr"/>
-      <c r="X78" s="3" t="inlineStr"/>
+      <c r="P78" s="3" t="n"/>
+      <c r="Q78" s="3" t="n"/>
+      <c r="R78" s="3" t="n"/>
+      <c r="S78" s="3" t="n"/>
+      <c r="T78" s="3" t="n"/>
+      <c r="U78" s="3" t="n"/>
+      <c r="V78" s="3" t="n"/>
+      <c r="W78" s="3" t="n"/>
+      <c r="X78" s="3" t="n"/>
       <c r="Y78" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -7820,7 +7820,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA78" s="3" t="inlineStr"/>
+      <c r="AA78" s="3" t="n"/>
       <c r="AB78" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -8177,15 +8177,15 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P82" s="3" t="inlineStr"/>
-      <c r="Q82" s="3" t="inlineStr"/>
-      <c r="R82" s="3" t="inlineStr"/>
-      <c r="S82" s="3" t="inlineStr"/>
-      <c r="T82" s="3" t="inlineStr"/>
-      <c r="U82" s="3" t="inlineStr"/>
-      <c r="V82" s="3" t="inlineStr"/>
-      <c r="W82" s="3" t="inlineStr"/>
-      <c r="X82" s="3" t="inlineStr"/>
+      <c r="P82" s="3" t="n"/>
+      <c r="Q82" s="3" t="n"/>
+      <c r="R82" s="3" t="n"/>
+      <c r="S82" s="3" t="n"/>
+      <c r="T82" s="3" t="n"/>
+      <c r="U82" s="3" t="n"/>
+      <c r="V82" s="3" t="n"/>
+      <c r="W82" s="3" t="n"/>
+      <c r="X82" s="3" t="n"/>
       <c r="Y82" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -8196,7 +8196,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA82" s="3" t="inlineStr"/>
+      <c r="AA82" s="3" t="n"/>
       <c r="AB82" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -8823,15 +8823,15 @@
       </c>
       <c r="N89" s="3" t="inlineStr"/>
       <c r="O89" s="3" t="inlineStr"/>
-      <c r="P89" s="3" t="inlineStr"/>
-      <c r="Q89" s="3" t="inlineStr"/>
-      <c r="R89" s="3" t="inlineStr"/>
-      <c r="S89" s="3" t="inlineStr"/>
-      <c r="T89" s="3" t="inlineStr"/>
-      <c r="U89" s="3" t="inlineStr"/>
-      <c r="V89" s="3" t="inlineStr"/>
-      <c r="W89" s="3" t="inlineStr"/>
-      <c r="X89" s="3" t="inlineStr"/>
+      <c r="P89" s="3" t="n"/>
+      <c r="Q89" s="3" t="n"/>
+      <c r="R89" s="3" t="n"/>
+      <c r="S89" s="3" t="n"/>
+      <c r="T89" s="3" t="n"/>
+      <c r="U89" s="3" t="n"/>
+      <c r="V89" s="3" t="n"/>
+      <c r="W89" s="3" t="n"/>
+      <c r="X89" s="3" t="n"/>
       <c r="Y89" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -8842,7 +8842,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA89" s="3" t="inlineStr"/>
+      <c r="AA89" s="3" t="n"/>
       <c r="AB89" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -9113,15 +9113,15 @@
           <t>abstract, full text</t>
         </is>
       </c>
-      <c r="P92" s="3" t="inlineStr"/>
-      <c r="Q92" s="3" t="inlineStr"/>
-      <c r="R92" s="3" t="inlineStr"/>
-      <c r="S92" s="3" t="inlineStr"/>
-      <c r="T92" s="3" t="inlineStr"/>
-      <c r="U92" s="3" t="inlineStr"/>
-      <c r="V92" s="3" t="inlineStr"/>
-      <c r="W92" s="3" t="inlineStr"/>
-      <c r="X92" s="3" t="inlineStr"/>
+      <c r="P92" s="3" t="n"/>
+      <c r="Q92" s="3" t="n"/>
+      <c r="R92" s="3" t="n"/>
+      <c r="S92" s="3" t="n"/>
+      <c r="T92" s="3" t="n"/>
+      <c r="U92" s="3" t="n"/>
+      <c r="V92" s="3" t="n"/>
+      <c r="W92" s="3" t="n"/>
+      <c r="X92" s="3" t="n"/>
       <c r="Y92" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -9132,7 +9132,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA92" s="3" t="inlineStr"/>
+      <c r="AA92" s="3" t="n"/>
       <c r="AB92" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -9497,18 +9497,18 @@
           <t>abstract, full text</t>
         </is>
       </c>
-      <c r="P96" s="3" t="inlineStr"/>
-      <c r="Q96" s="3" t="inlineStr"/>
-      <c r="R96" s="3" t="inlineStr"/>
-      <c r="S96" s="3" t="inlineStr"/>
-      <c r="T96" s="3" t="inlineStr"/>
-      <c r="U96" s="3" t="inlineStr"/>
-      <c r="V96" s="3" t="inlineStr"/>
-      <c r="W96" s="3" t="inlineStr"/>
-      <c r="X96" s="3" t="inlineStr"/>
+      <c r="P96" s="3" t="n"/>
+      <c r="Q96" s="3" t="n"/>
+      <c r="R96" s="3" t="n"/>
+      <c r="S96" s="3" t="n"/>
+      <c r="T96" s="3" t="n"/>
+      <c r="U96" s="3" t="n"/>
+      <c r="V96" s="3" t="n"/>
+      <c r="W96" s="3" t="n"/>
+      <c r="X96" s="3" t="n"/>
       <c r="Y96" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z96" s="3" t="inlineStr">
@@ -9516,7 +9516,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA96" s="3" t="inlineStr"/>
+      <c r="AA96" s="3" t="n"/>
       <c r="AB96" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -10155,15 +10155,15 @@
           <t>abstract, full text, recall</t>
         </is>
       </c>
-      <c r="P103" s="3" t="inlineStr"/>
-      <c r="Q103" s="3" t="inlineStr"/>
-      <c r="R103" s="3" t="inlineStr"/>
-      <c r="S103" s="3" t="inlineStr"/>
-      <c r="T103" s="3" t="inlineStr"/>
-      <c r="U103" s="3" t="inlineStr"/>
-      <c r="V103" s="3" t="inlineStr"/>
-      <c r="W103" s="3" t="inlineStr"/>
-      <c r="X103" s="3" t="inlineStr"/>
+      <c r="P103" s="3" t="n"/>
+      <c r="Q103" s="3" t="n"/>
+      <c r="R103" s="3" t="n"/>
+      <c r="S103" s="3" t="n"/>
+      <c r="T103" s="3" t="n"/>
+      <c r="U103" s="3" t="n"/>
+      <c r="V103" s="3" t="n"/>
+      <c r="W103" s="3" t="n"/>
+      <c r="X103" s="3" t="n"/>
       <c r="Y103" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -10174,7 +10174,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA103" s="3" t="inlineStr"/>
+      <c r="AA103" s="3" t="n"/>
       <c r="AB103" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -10911,15 +10911,15 @@
           <t>abstract, full text</t>
         </is>
       </c>
-      <c r="P111" s="3" t="inlineStr"/>
-      <c r="Q111" s="3" t="inlineStr"/>
-      <c r="R111" s="3" t="inlineStr"/>
-      <c r="S111" s="3" t="inlineStr"/>
-      <c r="T111" s="3" t="inlineStr"/>
-      <c r="U111" s="3" t="inlineStr"/>
-      <c r="V111" s="3" t="inlineStr"/>
-      <c r="W111" s="3" t="inlineStr"/>
-      <c r="X111" s="3" t="inlineStr"/>
+      <c r="P111" s="3" t="n"/>
+      <c r="Q111" s="3" t="n"/>
+      <c r="R111" s="3" t="n"/>
+      <c r="S111" s="3" t="n"/>
+      <c r="T111" s="3" t="n"/>
+      <c r="U111" s="3" t="n"/>
+      <c r="V111" s="3" t="n"/>
+      <c r="W111" s="3" t="n"/>
+      <c r="X111" s="3" t="n"/>
       <c r="Y111" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -10930,7 +10930,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA111" s="3" t="inlineStr"/>
+      <c r="AA111" s="3" t="n"/>
       <c r="AB111" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -11675,15 +11675,15 @@
           <t>abstract, full text</t>
         </is>
       </c>
-      <c r="P119" s="3" t="inlineStr"/>
-      <c r="Q119" s="3" t="inlineStr"/>
-      <c r="R119" s="3" t="inlineStr"/>
-      <c r="S119" s="3" t="inlineStr"/>
-      <c r="T119" s="3" t="inlineStr"/>
-      <c r="U119" s="3" t="inlineStr"/>
-      <c r="V119" s="3" t="inlineStr"/>
-      <c r="W119" s="3" t="inlineStr"/>
-      <c r="X119" s="3" t="inlineStr"/>
+      <c r="P119" s="3" t="n"/>
+      <c r="Q119" s="3" t="n"/>
+      <c r="R119" s="3" t="n"/>
+      <c r="S119" s="3" t="n"/>
+      <c r="T119" s="3" t="n"/>
+      <c r="U119" s="3" t="n"/>
+      <c r="V119" s="3" t="n"/>
+      <c r="W119" s="3" t="n"/>
+      <c r="X119" s="3" t="n"/>
       <c r="Y119" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -11694,7 +11694,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA119" s="3" t="inlineStr"/>
+      <c r="AA119" s="3" t="n"/>
       <c r="AB119" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -12533,15 +12533,15 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P128" s="3" t="inlineStr"/>
-      <c r="Q128" s="3" t="inlineStr"/>
-      <c r="R128" s="3" t="inlineStr"/>
-      <c r="S128" s="3" t="inlineStr"/>
-      <c r="T128" s="3" t="inlineStr"/>
-      <c r="U128" s="3" t="inlineStr"/>
-      <c r="V128" s="3" t="inlineStr"/>
-      <c r="W128" s="3" t="inlineStr"/>
-      <c r="X128" s="3" t="inlineStr"/>
+      <c r="P128" s="3" t="n"/>
+      <c r="Q128" s="3" t="n"/>
+      <c r="R128" s="3" t="n"/>
+      <c r="S128" s="3" t="n"/>
+      <c r="T128" s="3" t="n"/>
+      <c r="U128" s="3" t="n"/>
+      <c r="V128" s="3" t="n"/>
+      <c r="W128" s="3" t="n"/>
+      <c r="X128" s="3" t="n"/>
       <c r="Y128" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -12552,7 +12552,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA128" s="3" t="inlineStr"/>
+      <c r="AA128" s="3" t="n"/>
       <c r="AB128" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -12913,15 +12913,15 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P132" s="3" t="inlineStr"/>
-      <c r="Q132" s="3" t="inlineStr"/>
-      <c r="R132" s="3" t="inlineStr"/>
-      <c r="S132" s="3" t="inlineStr"/>
-      <c r="T132" s="3" t="inlineStr"/>
-      <c r="U132" s="3" t="inlineStr"/>
-      <c r="V132" s="3" t="inlineStr"/>
-      <c r="W132" s="3" t="inlineStr"/>
-      <c r="X132" s="3" t="inlineStr"/>
+      <c r="P132" s="3" t="n"/>
+      <c r="Q132" s="3" t="n"/>
+      <c r="R132" s="3" t="n"/>
+      <c r="S132" s="3" t="n"/>
+      <c r="T132" s="3" t="n"/>
+      <c r="U132" s="3" t="n"/>
+      <c r="V132" s="3" t="n"/>
+      <c r="W132" s="3" t="n"/>
+      <c r="X132" s="3" t="n"/>
       <c r="Y132" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -12932,7 +12932,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA132" s="3" t="inlineStr"/>
+      <c r="AA132" s="3" t="n"/>
       <c r="AB132" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -13297,18 +13297,18 @@
           <t>abstract, full text</t>
         </is>
       </c>
-      <c r="P136" s="3" t="inlineStr"/>
-      <c r="Q136" s="3" t="inlineStr"/>
-      <c r="R136" s="3" t="inlineStr"/>
-      <c r="S136" s="3" t="inlineStr"/>
-      <c r="T136" s="3" t="inlineStr"/>
-      <c r="U136" s="3" t="inlineStr"/>
-      <c r="V136" s="3" t="inlineStr"/>
-      <c r="W136" s="3" t="inlineStr"/>
-      <c r="X136" s="3" t="inlineStr"/>
+      <c r="P136" s="3" t="n"/>
+      <c r="Q136" s="3" t="n"/>
+      <c r="R136" s="3" t="n"/>
+      <c r="S136" s="3" t="n"/>
+      <c r="T136" s="3" t="n"/>
+      <c r="U136" s="3" t="n"/>
+      <c r="V136" s="3" t="n"/>
+      <c r="W136" s="3" t="n"/>
+      <c r="X136" s="3" t="n"/>
       <c r="Y136" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z136" s="3" t="inlineStr">
@@ -13316,7 +13316,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA136" s="3" t="inlineStr"/>
+      <c r="AA136" s="3" t="n"/>
       <c r="AB136" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -13489,18 +13489,18 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P138" s="3" t="inlineStr"/>
-      <c r="Q138" s="3" t="inlineStr"/>
-      <c r="R138" s="3" t="inlineStr"/>
-      <c r="S138" s="3" t="inlineStr"/>
-      <c r="T138" s="3" t="inlineStr"/>
-      <c r="U138" s="3" t="inlineStr"/>
-      <c r="V138" s="3" t="inlineStr"/>
-      <c r="W138" s="3" t="inlineStr"/>
-      <c r="X138" s="3" t="inlineStr"/>
+      <c r="P138" s="3" t="n"/>
+      <c r="Q138" s="3" t="n"/>
+      <c r="R138" s="3" t="n"/>
+      <c r="S138" s="3" t="n"/>
+      <c r="T138" s="3" t="n"/>
+      <c r="U138" s="3" t="n"/>
+      <c r="V138" s="3" t="n"/>
+      <c r="W138" s="3" t="n"/>
+      <c r="X138" s="3" t="n"/>
       <c r="Y138" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z138" s="3" t="inlineStr">
@@ -13508,7 +13508,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA138" s="3" t="inlineStr"/>
+      <c r="AA138" s="3" t="n"/>
       <c r="AB138" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -13583,18 +13583,18 @@
           <t>full text</t>
         </is>
       </c>
-      <c r="P139" s="3" t="inlineStr"/>
-      <c r="Q139" s="3" t="inlineStr"/>
-      <c r="R139" s="3" t="inlineStr"/>
-      <c r="S139" s="3" t="inlineStr"/>
-      <c r="T139" s="3" t="inlineStr"/>
-      <c r="U139" s="3" t="inlineStr"/>
-      <c r="V139" s="3" t="inlineStr"/>
-      <c r="W139" s="3" t="inlineStr"/>
-      <c r="X139" s="3" t="inlineStr"/>
+      <c r="P139" s="3" t="n"/>
+      <c r="Q139" s="3" t="n"/>
+      <c r="R139" s="3" t="n"/>
+      <c r="S139" s="3" t="n"/>
+      <c r="T139" s="3" t="n"/>
+      <c r="U139" s="3" t="n"/>
+      <c r="V139" s="3" t="n"/>
+      <c r="W139" s="3" t="n"/>
+      <c r="X139" s="3" t="n"/>
       <c r="Y139" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z139" s="3" t="inlineStr">
@@ -13602,7 +13602,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA139" s="3" t="inlineStr"/>
+      <c r="AA139" s="3" t="n"/>
       <c r="AB139" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -13775,15 +13775,15 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P141" s="3" t="inlineStr"/>
-      <c r="Q141" s="3" t="inlineStr"/>
-      <c r="R141" s="3" t="inlineStr"/>
-      <c r="S141" s="3" t="inlineStr"/>
-      <c r="T141" s="3" t="inlineStr"/>
-      <c r="U141" s="3" t="inlineStr"/>
-      <c r="V141" s="3" t="inlineStr"/>
-      <c r="W141" s="3" t="inlineStr"/>
-      <c r="X141" s="3" t="inlineStr"/>
+      <c r="P141" s="3" t="n"/>
+      <c r="Q141" s="3" t="n"/>
+      <c r="R141" s="3" t="n"/>
+      <c r="S141" s="3" t="n"/>
+      <c r="T141" s="3" t="n"/>
+      <c r="U141" s="3" t="n"/>
+      <c r="V141" s="3" t="n"/>
+      <c r="W141" s="3" t="n"/>
+      <c r="X141" s="3" t="n"/>
       <c r="Y141" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -13794,7 +13794,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA141" s="3" t="inlineStr"/>
+      <c r="AA141" s="3" t="n"/>
       <c r="AB141" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -14065,18 +14065,18 @@
           <t>abstract, full text</t>
         </is>
       </c>
-      <c r="P144" s="3" t="inlineStr"/>
-      <c r="Q144" s="3" t="inlineStr"/>
-      <c r="R144" s="3" t="inlineStr"/>
-      <c r="S144" s="3" t="inlineStr"/>
-      <c r="T144" s="3" t="inlineStr"/>
-      <c r="U144" s="3" t="inlineStr"/>
-      <c r="V144" s="3" t="inlineStr"/>
-      <c r="W144" s="3" t="inlineStr"/>
-      <c r="X144" s="3" t="inlineStr"/>
+      <c r="P144" s="3" t="n"/>
+      <c r="Q144" s="3" t="n"/>
+      <c r="R144" s="3" t="n"/>
+      <c r="S144" s="3" t="n"/>
+      <c r="T144" s="3" t="n"/>
+      <c r="U144" s="3" t="n"/>
+      <c r="V144" s="3" t="n"/>
+      <c r="W144" s="3" t="n"/>
+      <c r="X144" s="3" t="n"/>
       <c r="Y144" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z144" s="3" t="inlineStr">
@@ -14084,7 +14084,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA144" s="3" t="inlineStr"/>
+      <c r="AA144" s="3" t="n"/>
       <c r="AB144" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -14837,18 +14837,18 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P152" s="3" t="inlineStr"/>
-      <c r="Q152" s="3" t="inlineStr"/>
-      <c r="R152" s="3" t="inlineStr"/>
-      <c r="S152" s="3" t="inlineStr"/>
-      <c r="T152" s="3" t="inlineStr"/>
-      <c r="U152" s="3" t="inlineStr"/>
-      <c r="V152" s="3" t="inlineStr"/>
-      <c r="W152" s="3" t="inlineStr"/>
-      <c r="X152" s="3" t="inlineStr"/>
+      <c r="P152" s="3" t="n"/>
+      <c r="Q152" s="3" t="n"/>
+      <c r="R152" s="3" t="n"/>
+      <c r="S152" s="3" t="n"/>
+      <c r="T152" s="3" t="n"/>
+      <c r="U152" s="3" t="n"/>
+      <c r="V152" s="3" t="n"/>
+      <c r="W152" s="3" t="n"/>
+      <c r="X152" s="3" t="n"/>
       <c r="Y152" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z152" s="3" t="inlineStr">
@@ -14856,7 +14856,7 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="AA152" s="3" t="inlineStr"/>
+      <c r="AA152" s="3" t="n"/>
       <c r="AB152" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -15119,18 +15119,18 @@
           <t>full text</t>
         </is>
       </c>
-      <c r="P155" s="3" t="inlineStr"/>
-      <c r="Q155" s="3" t="inlineStr"/>
-      <c r="R155" s="3" t="inlineStr"/>
-      <c r="S155" s="3" t="inlineStr"/>
-      <c r="T155" s="3" t="inlineStr"/>
-      <c r="U155" s="3" t="inlineStr"/>
-      <c r="V155" s="3" t="inlineStr"/>
-      <c r="W155" s="3" t="inlineStr"/>
-      <c r="X155" s="3" t="inlineStr"/>
+      <c r="P155" s="3" t="n"/>
+      <c r="Q155" s="3" t="n"/>
+      <c r="R155" s="3" t="n"/>
+      <c r="S155" s="3" t="n"/>
+      <c r="T155" s="3" t="n"/>
+      <c r="U155" s="3" t="n"/>
+      <c r="V155" s="3" t="n"/>
+      <c r="W155" s="3" t="n"/>
+      <c r="X155" s="3" t="n"/>
       <c r="Y155" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z155" s="3" t="inlineStr">
@@ -15138,7 +15138,7 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="AA155" s="3" t="inlineStr"/>
+      <c r="AA155" s="3" t="n"/>
       <c r="AB155" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -15209,15 +15209,15 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P156" s="3" t="inlineStr"/>
-      <c r="Q156" s="3" t="inlineStr"/>
-      <c r="R156" s="3" t="inlineStr"/>
-      <c r="S156" s="3" t="inlineStr"/>
-      <c r="T156" s="3" t="inlineStr"/>
-      <c r="U156" s="3" t="inlineStr"/>
-      <c r="V156" s="3" t="inlineStr"/>
-      <c r="W156" s="3" t="inlineStr"/>
-      <c r="X156" s="3" t="inlineStr"/>
+      <c r="P156" s="3" t="n"/>
+      <c r="Q156" s="3" t="n"/>
+      <c r="R156" s="3" t="n"/>
+      <c r="S156" s="3" t="n"/>
+      <c r="T156" s="3" t="n"/>
+      <c r="U156" s="3" t="n"/>
+      <c r="V156" s="3" t="n"/>
+      <c r="W156" s="3" t="n"/>
+      <c r="X156" s="3" t="n"/>
       <c r="Y156" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -15228,7 +15228,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA156" s="3" t="inlineStr"/>
+      <c r="AA156" s="3" t="n"/>
       <c r="AB156" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -15785,18 +15785,18 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P162" s="3" t="inlineStr"/>
-      <c r="Q162" s="3" t="inlineStr"/>
-      <c r="R162" s="3" t="inlineStr"/>
-      <c r="S162" s="3" t="inlineStr"/>
-      <c r="T162" s="3" t="inlineStr"/>
-      <c r="U162" s="3" t="inlineStr"/>
-      <c r="V162" s="3" t="inlineStr"/>
-      <c r="W162" s="3" t="inlineStr"/>
-      <c r="X162" s="3" t="inlineStr"/>
+      <c r="P162" s="3" t="n"/>
+      <c r="Q162" s="3" t="n"/>
+      <c r="R162" s="3" t="n"/>
+      <c r="S162" s="3" t="n"/>
+      <c r="T162" s="3" t="n"/>
+      <c r="U162" s="3" t="n"/>
+      <c r="V162" s="3" t="n"/>
+      <c r="W162" s="3" t="n"/>
+      <c r="X162" s="3" t="n"/>
       <c r="Y162" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z162" s="3" t="inlineStr">
@@ -15804,7 +15804,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA162" s="3" t="inlineStr"/>
+      <c r="AA162" s="3" t="n"/>
       <c r="AB162" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -16349,15 +16349,15 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P168" s="3" t="inlineStr"/>
-      <c r="Q168" s="3" t="inlineStr"/>
-      <c r="R168" s="3" t="inlineStr"/>
-      <c r="S168" s="3" t="inlineStr"/>
-      <c r="T168" s="3" t="inlineStr"/>
-      <c r="U168" s="3" t="inlineStr"/>
-      <c r="V168" s="3" t="inlineStr"/>
-      <c r="W168" s="3" t="inlineStr"/>
-      <c r="X168" s="3" t="inlineStr"/>
+      <c r="P168" s="3" t="n"/>
+      <c r="Q168" s="3" t="n"/>
+      <c r="R168" s="3" t="n"/>
+      <c r="S168" s="3" t="n"/>
+      <c r="T168" s="3" t="n"/>
+      <c r="U168" s="3" t="n"/>
+      <c r="V168" s="3" t="n"/>
+      <c r="W168" s="3" t="n"/>
+      <c r="X168" s="3" t="n"/>
       <c r="Y168" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -16368,7 +16368,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA168" s="3" t="inlineStr"/>
+      <c r="AA168" s="3" t="n"/>
       <c r="AB168" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -16443,15 +16443,15 @@
           <t>abstract, full text</t>
         </is>
       </c>
-      <c r="P169" s="3" t="inlineStr"/>
-      <c r="Q169" s="3" t="inlineStr"/>
-      <c r="R169" s="3" t="inlineStr"/>
-      <c r="S169" s="3" t="inlineStr"/>
-      <c r="T169" s="3" t="inlineStr"/>
-      <c r="U169" s="3" t="inlineStr"/>
-      <c r="V169" s="3" t="inlineStr"/>
-      <c r="W169" s="3" t="inlineStr"/>
-      <c r="X169" s="3" t="inlineStr"/>
+      <c r="P169" s="3" t="n"/>
+      <c r="Q169" s="3" t="n"/>
+      <c r="R169" s="3" t="n"/>
+      <c r="S169" s="3" t="n"/>
+      <c r="T169" s="3" t="n"/>
+      <c r="U169" s="3" t="n"/>
+      <c r="V169" s="3" t="n"/>
+      <c r="W169" s="3" t="n"/>
+      <c r="X169" s="3" t="n"/>
       <c r="Y169" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -16462,7 +16462,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA169" s="3" t="inlineStr"/>
+      <c r="AA169" s="3" t="n"/>
       <c r="AB169" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -16631,18 +16631,18 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P171" s="3" t="inlineStr"/>
-      <c r="Q171" s="3" t="inlineStr"/>
-      <c r="R171" s="3" t="inlineStr"/>
-      <c r="S171" s="3" t="inlineStr"/>
-      <c r="T171" s="3" t="inlineStr"/>
-      <c r="U171" s="3" t="inlineStr"/>
-      <c r="V171" s="3" t="inlineStr"/>
-      <c r="W171" s="3" t="inlineStr"/>
-      <c r="X171" s="3" t="inlineStr"/>
+      <c r="P171" s="3" t="n"/>
+      <c r="Q171" s="3" t="n"/>
+      <c r="R171" s="3" t="n"/>
+      <c r="S171" s="3" t="n"/>
+      <c r="T171" s="3" t="n"/>
+      <c r="U171" s="3" t="n"/>
+      <c r="V171" s="3" t="n"/>
+      <c r="W171" s="3" t="n"/>
+      <c r="X171" s="3" t="n"/>
       <c r="Y171" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z171" s="3" t="inlineStr">
@@ -16650,7 +16650,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA171" s="3" t="inlineStr"/>
+      <c r="AA171" s="3" t="n"/>
       <c r="AB171" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -17117,18 +17117,18 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="P176" s="3" t="inlineStr"/>
-      <c r="Q176" s="3" t="inlineStr"/>
-      <c r="R176" s="3" t="inlineStr"/>
-      <c r="S176" s="3" t="inlineStr"/>
-      <c r="T176" s="3" t="inlineStr"/>
-      <c r="U176" s="3" t="inlineStr"/>
-      <c r="V176" s="3" t="inlineStr"/>
-      <c r="W176" s="3" t="inlineStr"/>
-      <c r="X176" s="3" t="inlineStr"/>
+      <c r="P176" s="3" t="n"/>
+      <c r="Q176" s="3" t="n"/>
+      <c r="R176" s="3" t="n"/>
+      <c r="S176" s="3" t="n"/>
+      <c r="T176" s="3" t="n"/>
+      <c r="U176" s="3" t="n"/>
+      <c r="V176" s="3" t="n"/>
+      <c r="W176" s="3" t="n"/>
+      <c r="X176" s="3" t="n"/>
       <c r="Y176" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z176" s="3" t="inlineStr">
@@ -17136,7 +17136,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA176" s="3" t="inlineStr"/>
+      <c r="AA176" s="3" t="n"/>
       <c r="AB176" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -17399,18 +17399,18 @@
           <t>full text</t>
         </is>
       </c>
-      <c r="P179" s="3" t="inlineStr"/>
-      <c r="Q179" s="3" t="inlineStr"/>
-      <c r="R179" s="3" t="inlineStr"/>
-      <c r="S179" s="3" t="inlineStr"/>
-      <c r="T179" s="3" t="inlineStr"/>
-      <c r="U179" s="3" t="inlineStr"/>
-      <c r="V179" s="3" t="inlineStr"/>
-      <c r="W179" s="3" t="inlineStr"/>
-      <c r="X179" s="3" t="inlineStr"/>
+      <c r="P179" s="3" t="n"/>
+      <c r="Q179" s="3" t="n"/>
+      <c r="R179" s="3" t="n"/>
+      <c r="S179" s="3" t="n"/>
+      <c r="T179" s="3" t="n"/>
+      <c r="U179" s="3" t="n"/>
+      <c r="V179" s="3" t="n"/>
+      <c r="W179" s="3" t="n"/>
+      <c r="X179" s="3" t="n"/>
       <c r="Y179" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>txt</t>
         </is>
       </c>
       <c r="Z179" s="3" t="inlineStr">
@@ -17418,7 +17418,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="AA179" s="3" t="inlineStr"/>
+      <c r="AA179" s="3" t="n"/>
       <c r="AB179" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>

</xml_diff>

<commit_message>
Track open-access locations for corpus articles without a local text; download the 8 reachable PDFs
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/corpus/corpus.xlsx
+++ b/corpus/corpus.xlsx
@@ -6210,7 +6210,7 @@
       <c r="X61" s="3" t="n"/>
       <c r="Y61" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z61" s="3" t="inlineStr">
@@ -8560,7 +8560,7 @@
       <c r="X86" s="3" t="n"/>
       <c r="Y86" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z86" s="3" t="inlineStr">
@@ -9970,7 +9970,7 @@
       <c r="X101" s="3" t="n"/>
       <c r="Y101" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z101" s="3" t="inlineStr">
@@ -12638,7 +12638,7 @@
       <c r="X129" s="3" t="n"/>
       <c r="Y129" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z129" s="3" t="inlineStr">
@@ -14264,7 +14264,7 @@
       <c r="X146" s="3" t="n"/>
       <c r="Y146" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z146" s="3" t="inlineStr">
@@ -14938,7 +14938,7 @@
       <c r="X153" s="3" t="n"/>
       <c r="Y153" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z153" s="3" t="inlineStr">
@@ -16454,7 +16454,7 @@
       <c r="X169" s="3" t="n"/>
       <c r="Y169" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z169" s="3" t="inlineStr">
@@ -17888,7 +17888,7 @@
       <c r="X184" s="3" t="n"/>
       <c r="Y184" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z184" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Daily watch 2026-10-27: 6 records, 2 candidates, 0 entries, urgent=no
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/corpus/corpus.xlsx
+++ b/corpus/corpus.xlsx
@@ -688,7 +688,7 @@
       <c r="X2" s="3" t="n"/>
       <c r="Y2" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z2" s="3" t="inlineStr">
@@ -1424,7 +1424,7 @@
       <c r="X8" s="3" t="n"/>
       <c r="Y8" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z8" s="3" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>abstract, full text, title only</t>
+          <t>abstract, full text</t>
         </is>
       </c>
       <c r="P9" s="3" t="n"/>
@@ -1836,7 +1836,7 @@
       <c r="X12" s="3" t="n"/>
       <c r="Y12" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z12" s="3" t="inlineStr">
@@ -1926,7 +1926,7 @@
       <c r="X13" s="3" t="n"/>
       <c r="Y13" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z13" s="3" t="inlineStr">
@@ -2146,7 +2146,7 @@
       <c r="X15" s="3" t="n"/>
       <c r="Y15" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z15" s="3" t="inlineStr">
@@ -2226,7 +2226,7 @@
       </c>
       <c r="O16" s="3" t="inlineStr">
         <is>
-          <t>abstract, full text, title only</t>
+          <t>abstract, full text</t>
         </is>
       </c>
       <c r="P16" s="3" t="n"/>
@@ -2460,7 +2460,7 @@
       <c r="X18" s="3" t="n"/>
       <c r="Y18" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z18" s="3" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>abstract, full text, title only</t>
+          <t>abstract, full text</t>
         </is>
       </c>
       <c r="P20" s="3" t="n"/>
@@ -2778,7 +2778,7 @@
       <c r="X21" s="3" t="n"/>
       <c r="Y21" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z21" s="3" t="inlineStr">
@@ -3116,12 +3116,12 @@
       <c r="L24" s="3" t="inlineStr"/>
       <c r="M24" s="3" t="inlineStr">
         <is>
-          <t>U1: text; U6: text; V10: text; V11: text; V12: text; V13: text; V14: text; V19: text; V1: text; V20: text; V23: text; V24: text; V25: text; V2: text; V4: text; V6: text; V8: text; V9: text; usecases-verified: row 1; usecases-verified: row 48</t>
+          <t>U1: text; U6: text; V10: text; V11: text; V12: text; V13: text; V14: text; V19: text; V1: text; V20: text; V23: text; V24: text; V25: text; V2: text; V4: text; V6: text; V8: text; V9: text; usecases-verified: row 1; usecases-verified: row 23; usecases-verified: row 48</t>
         </is>
       </c>
       <c r="N24" s="3" t="inlineStr">
         <is>
-          <t>1,48</t>
+          <t>1,23,48</t>
         </is>
       </c>
       <c r="O24" s="3" t="inlineStr">
@@ -3230,7 +3230,7 @@
       <c r="X25" s="3" t="n"/>
       <c r="Y25" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z25" s="3" t="inlineStr">
@@ -4236,12 +4236,12 @@
       <c r="L34" s="3" t="inlineStr"/>
       <c r="M34" s="3" t="inlineStr">
         <is>
-          <t>V2: text; V3: text; V4: text; usecases-verified: row 7</t>
+          <t>V2: text; V3: text; V4: text; usecases-verified: row 33; usecases-verified: row 7</t>
         </is>
       </c>
       <c r="N34" s="3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>7,33</t>
         </is>
       </c>
       <c r="O34" s="3" t="inlineStr">
@@ -5006,7 +5006,7 @@
       <c r="X41" s="3" t="n"/>
       <c r="Y41" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z41" s="3" t="inlineStr">
@@ -5284,7 +5284,7 @@
       <c r="X44" s="3" t="n"/>
       <c r="Y44" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z44" s="3" t="inlineStr">
@@ -5798,7 +5798,7 @@
       <c r="L49" s="3" t="inlineStr"/>
       <c r="M49" s="3" t="inlineStr">
         <is>
-          <t>U2: text; U3: text; U4: text; U5: text; U6: text; V14: text; V15: text; V16: text; V17: text; V18: text; V19: text; V2: text; V4: text; usecases-verified: row 28; usecases-verified: row 6</t>
+          <t>U2: text; U3: text; U4: text; U5: text; U6: text; V14: text; V15: text; V16: text; V17: text; V18: text; V19: text; V2: text; V3: text; V4: text; usecases-verified: row 28; usecases-verified: row 6</t>
         </is>
       </c>
       <c r="N49" s="3" t="inlineStr">
@@ -6186,7 +6186,7 @@
       <c r="X53" s="3" t="n"/>
       <c r="Y53" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z53" s="3" t="inlineStr">
@@ -7144,7 +7144,7 @@
       <c r="X62" s="3" t="n"/>
       <c r="Y62" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z62" s="3" t="inlineStr">
@@ -7234,7 +7234,7 @@
       <c r="X63" s="3" t="n"/>
       <c r="Y63" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z63" s="3" t="inlineStr">
@@ -8336,7 +8336,7 @@
       <c r="X74" s="3" t="n"/>
       <c r="Y74" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z74" s="3" t="inlineStr">
@@ -8524,7 +8524,7 @@
       <c r="X76" s="3" t="n"/>
       <c r="Y76" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z76" s="3" t="inlineStr">
@@ -8748,7 +8748,7 @@
       <c r="X78" s="3" t="n"/>
       <c r="Y78" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z78" s="3" t="inlineStr">
@@ -8916,12 +8916,12 @@
       <c r="L80" s="3" t="inlineStr"/>
       <c r="M80" s="3" t="inlineStr">
         <is>
-          <t>V10: text; V11: text; V12: text; V13: text; V8: text; V9: text; usecases-verified: row 1; usecases-verified: row 22</t>
+          <t>V10: text; V11: text; V12: text; V13: text; V8: text; V9: text; usecases-verified: row 1; usecases-verified: row 22; usecases-verified: row 23</t>
         </is>
       </c>
       <c r="N80" s="3" t="inlineStr">
         <is>
-          <t>1,22</t>
+          <t>1,22,23</t>
         </is>
       </c>
       <c r="O80" s="3" t="inlineStr">
@@ -9124,7 +9124,7 @@
       <c r="X82" s="3" t="n"/>
       <c r="Y82" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z82" s="3" t="inlineStr">
@@ -9984,7 +9984,7 @@
       <c r="X90" s="3" t="n"/>
       <c r="Y90" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z90" s="3" t="inlineStr">
@@ -10446,7 +10446,7 @@
       <c r="X95" s="3" t="n"/>
       <c r="Y95" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z95" s="3" t="inlineStr">
@@ -13040,7 +13040,7 @@
       <c r="X120" s="3" t="n"/>
       <c r="Y120" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z120" s="3" t="inlineStr">
@@ -13506,7 +13506,7 @@
       <c r="X125" s="3" t="n"/>
       <c r="Y125" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z125" s="3" t="inlineStr">
@@ -13596,7 +13596,7 @@
       <c r="X126" s="3" t="n"/>
       <c r="Y126" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z126" s="3" t="inlineStr">
@@ -13878,7 +13878,7 @@
       <c r="X129" s="3" t="n"/>
       <c r="Y129" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z129" s="3" t="inlineStr">
@@ -14568,7 +14568,7 @@
       <c r="X136" s="3" t="n"/>
       <c r="Y136" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z136" s="3" t="inlineStr">
@@ -14826,12 +14826,12 @@
       <c r="L139" s="3" t="inlineStr"/>
       <c r="M139" s="3" t="inlineStr">
         <is>
-          <t>V11: text; V12: text; V13: text; V3: text; V4: text; V9: text; usecases-verified: row 33; usecases-verified: row 7</t>
+          <t>V11: text; V12: text; V13: text; V3: text; V4: text; V9: text; usecases-verified: row 33</t>
         </is>
       </c>
       <c r="N139" s="3" t="inlineStr">
         <is>
-          <t>7,33</t>
+          <t>33</t>
         </is>
       </c>
       <c r="O139" s="3" t="inlineStr">
@@ -15742,7 +15742,7 @@
       <c r="X147" s="3" t="n"/>
       <c r="Y147" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z147" s="3" t="inlineStr">
@@ -16004,12 +16004,12 @@
       <c r="L150" s="3" t="inlineStr"/>
       <c r="M150" s="3" t="inlineStr">
         <is>
-          <t>U4: text; V1: text; usecases-verified: row 6</t>
+          <t>U4: text; V1: text; usecases-verified: row 47; usecases-verified: row 6</t>
         </is>
       </c>
       <c r="N150" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>6,47</t>
         </is>
       </c>
       <c r="O150" s="3" t="inlineStr">
@@ -16460,13 +16460,17 @@
       <c r="L154" s="3" t="inlineStr"/>
       <c r="M154" s="3" t="inlineStr">
         <is>
-          <t>V2: text</t>
-        </is>
-      </c>
-      <c r="N154" s="3" t="inlineStr"/>
+          <t>V2: text; usecases-verified: row 10</t>
+        </is>
+      </c>
+      <c r="N154" s="3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="O154" s="3" t="inlineStr">
         <is>
-          <t>abstract, full text</t>
+          <t>abstract, full text, recall</t>
         </is>
       </c>
       <c r="P154" s="3" t="n"/>
@@ -16856,7 +16860,7 @@
       <c r="X158" s="3" t="n"/>
       <c r="Y158" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z158" s="3" t="inlineStr">
@@ -17750,7 +17754,7 @@
       <c r="X167" s="3" t="n"/>
       <c r="Y167" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z167" s="3" t="inlineStr">
@@ -17840,7 +17844,7 @@
       <c r="X168" s="3" t="n"/>
       <c r="Y168" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z168" s="3" t="inlineStr">
@@ -18256,7 +18260,7 @@
       <c r="X172" s="3" t="n"/>
       <c r="Y172" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z172" s="3" t="inlineStr">
@@ -18958,7 +18962,7 @@
       <c r="X179" s="3" t="n"/>
       <c r="Y179" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z179" s="3" t="inlineStr">
@@ -20582,7 +20586,7 @@
       <c r="X195" s="3" t="n"/>
       <c r="Y195" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z195" s="3" t="inlineStr">
@@ -20868,7 +20872,7 @@
       <c r="X198" s="3" t="n"/>
       <c r="Y198" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z198" s="3" t="inlineStr">
@@ -21624,7 +21628,7 @@
       <c r="X206" s="3" t="n"/>
       <c r="Y206" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z206" s="3" t="inlineStr">
@@ -22380,7 +22384,7 @@
       <c r="X214" s="3" t="n"/>
       <c r="Y214" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z214" s="3" t="inlineStr">
@@ -22972,7 +22976,7 @@
       <c r="X220" s="3" t="n"/>
       <c r="Y220" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z220" s="3" t="inlineStr">
@@ -23580,7 +23584,7 @@
       <c r="X226" s="3" t="n"/>
       <c r="Y226" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z226" s="3" t="inlineStr">
@@ -23670,7 +23674,7 @@
       <c r="X227" s="3" t="n"/>
       <c r="Y227" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z227" s="3" t="inlineStr">
@@ -24858,7 +24862,7 @@
       <c r="X239" s="3" t="n"/>
       <c r="Y239" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z239" s="3" t="inlineStr">
@@ -28402,7 +28406,7 @@
       <c r="X275" s="3" t="n"/>
       <c r="Y275" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z275" s="3" t="inlineStr">
@@ -28766,7 +28770,7 @@
       <c r="X279" s="3" t="n"/>
       <c r="Y279" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z279" s="3" t="inlineStr">
@@ -30288,7 +30292,7 @@
       <c r="X294" s="3" t="n"/>
       <c r="Y294" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z294" s="3" t="inlineStr">
@@ -32378,7 +32382,7 @@
       <c r="X315" s="3" t="n"/>
       <c r="Y315" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z315" s="3" t="inlineStr">
@@ -34088,7 +34092,7 @@
       <c r="X330" s="3" t="n"/>
       <c r="Y330" s="3" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="Z330" s="3" t="inlineStr">

</xml_diff>